<commit_message>
Rendiconto e report: contatori bloccati MG5/MG8/MG6, profilo giorno/notte, benchmark servizi
</commit_message>
<xml_diff>
--- a/rendiconto_2025_2026.xlsx
+++ b/rendiconto_2025_2026.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1130,115 +1130,100 @@
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>12. Contatori con trasmissione interrotta. MG5 e MG8 (dal 14/05/2026) e MG6 (dall'11/05/2026) risultano in produzione ma il rispettivo contatore IcoPower non aggiorna piu: i kWh 2026 di queste macchine sono SOTTOSTIMATI (l'ultima lettura valida e di maggio). Ore e pezzi restano validi (fonti ProdWare/turni). Dove intervenire: rilevatore/trasmissione dei tre contatori (vedi report Direttore di Produzione).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
         <is>
           <t>5. CONSISTENZA DATI (CROSS-CHECK)</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
         <is>
           <t>Indicatore</t>
         </is>
       </c>
-      <c r="B58" s="4" t="inlineStr">
+      <c r="B59" s="4" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
+      <c r="C59" s="4" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr">
+      <c r="D59" s="4" t="inlineStr">
         <is>
           <t>Fonte</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>kWh misurati IcoPower</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>147.103 (GEN-NOV)</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>72.467 (GEN-SET)</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>IcoPower / consolidato</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>kWh bollettati ENEL</t>
+          <t>kWh misurati IcoPower</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>500.743 (GEN-NOV)</t>
+          <t>147.103 (GEN-NOV)</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>396.200 (DIC25-LUG26)</t>
+          <t>72.467 (GEN-SET)</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Fatture ENEL</t>
+          <t>IcoPower / consolidato</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>Ore lavoro ODL</t>
+          <t>kWh bollettati ENEL</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>20.624</t>
+          <t>500.743 (GEN-NOV)</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>12.186</t>
+          <t>396.200 (DIC25-LUG26)</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>ProdWare ODL</t>
+          <t>Fatture ENEL</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>Ore fermo ODL</t>
+          <t>Ore lavoro ODL</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>30.928</t>
+          <t>20.624</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>15.560</t>
+          <t>12.186</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
@@ -1250,75 +1235,97 @@
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>Ore lavoro file turni</t>
+          <t>Ore fermo ODL</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>20.624 (GEN-DIC)</t>
+          <t>30.928</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>12.235 (GEN-SET)</t>
+          <t>15.560</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>File turni</t>
+          <t>ProdWare ODL</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
+          <t>Ore lavoro file turni</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>20.624 (GEN-DIC)</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>12.235 (GEN-SET)</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>File turni</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
           <t>Pezzi (esclusa N/A)</t>
         </is>
       </c>
-      <c r="B64" s="5" t="inlineStr">
+      <c r="B65" s="5" t="inlineStr">
         <is>
           <t>7.931.600</t>
         </is>
       </c>
-      <c r="C64" s="5" t="inlineStr">
+      <c r="C65" s="5" t="inlineStr">
         <is>
           <t>4.122.557</t>
         </is>
       </c>
-      <c r="D64" s="5" t="inlineStr">
+      <c r="D65" s="5" t="inlineStr">
         <is>
           <t>ProdWare Qta / Tabelle</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
         <is>
           <t>6. NOTE FINALI</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="6" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
         <is>
           <t>Elaborazione a cura di ZetaByteNexus. Dati estratti dai sistemi aziendali (IcoPower, ProdWare) e dalle bollette ENEL allegate in input/. Il confronto 2025/2026 e pensato per l'analisi dei consumi e dell'efficienza energetica per macchina. Per aggiornamenti o chiarimenti rivolgersi al referente tecnico.</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="6" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
         <is>
           <t>Versione 2.0 | 14/09/2026 | Sostituisce la versione 1.0 (solo 2026)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
     <mergeCell ref="A45:D45"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A67:D67"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="A70:D70"/>
     <mergeCell ref="A53:D53"/>
-    <mergeCell ref="A69:D69"/>
     <mergeCell ref="A50:D50"/>
     <mergeCell ref="A48:D48"/>
     <mergeCell ref="A3:D3"/>
@@ -1330,6 +1337,7 @@
     <mergeCell ref="A49:D49"/>
     <mergeCell ref="A47:D47"/>
     <mergeCell ref="A46:D46"/>
+    <mergeCell ref="A68:D68"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12298,7 +12306,11 @@
       <c r="J24" s="12" t="n">
         <v>19.31</v>
       </c>
-      <c r="K24" s="9" t="inlineStr"/>
+      <c r="K24" s="9" t="inlineStr">
+        <is>
+          <t>dato incompleto: contatore fermo dal 14/05/2026 (macchina in produzione)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
@@ -12333,7 +12345,11 @@
       <c r="J25" s="12" t="n">
         <v>-61.22</v>
       </c>
-      <c r="K25" s="9" t="inlineStr"/>
+      <c r="K25" s="9" t="inlineStr">
+        <is>
+          <t>dato incompleto: contatore fermo dall'11/05/2026 (macchina in produzione)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
@@ -12403,7 +12419,11 @@
       <c r="J27" s="12" t="n">
         <v>-6.22</v>
       </c>
-      <c r="K27" s="9" t="inlineStr"/>
+      <c r="K27" s="9" t="inlineStr">
+        <is>
+          <t>dato incompleto: contatore fermo dal 14/05/2026 (macchina in produzione)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
@@ -14335,7 +14355,11 @@
       <c r="L19" s="11" t="n">
         <v>428.0705897169485</v>
       </c>
-      <c r="M19" s="9" t="inlineStr"/>
+      <c r="M19" s="9" t="inlineStr">
+        <is>
+          <t>dato incompleto: contatore fermo dal 14/05/2026 (macchina in produzione)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -14376,7 +14400,11 @@
       <c r="L20" s="11" t="n">
         <v>305.6168734317149</v>
       </c>
-      <c r="M20" s="9" t="inlineStr"/>
+      <c r="M20" s="9" t="inlineStr">
+        <is>
+          <t>dato incompleto: contatore fermo dall'11/05/2026 (macchina in produzione)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
@@ -14458,7 +14486,11 @@
       <c r="L22" s="11" t="n">
         <v>126.0466646249475</v>
       </c>
-      <c r="M22" s="9" t="inlineStr"/>
+      <c r="M22" s="9" t="inlineStr">
+        <is>
+          <t>dato incompleto: contatore fermo dal 14/05/2026 (macchina in produzione)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">

</xml_diff>